<commit_message>
Integrate tested draw.io library with current grounded evidence and report review
</commit_message>
<xml_diff>
--- a/generated/logic/08_TAG_LOGIC_LINK_MASTER_VALIDATION.xlsx
+++ b/generated/logic/08_TAG_LOGIC_LINK_MASTER_VALIDATION.xlsx
@@ -81,7 +81,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">603</t>
+          <t xml:space="preserve">604</t>
         </is>
       </c>
     </row>
@@ -93,7 +93,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">53</t>
+          <t xml:space="preserve">54</t>
         </is>
       </c>
     </row>
@@ -105,7 +105,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">35</t>
+          <t xml:space="preserve">36</t>
         </is>
       </c>
     </row>
@@ -129,7 +129,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">98</t>
+          <t xml:space="preserve">100</t>
         </is>
       </c>
     </row>
@@ -141,7 +141,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">44</t>
+          <t xml:space="preserve">45</t>
         </is>
       </c>
     </row>
@@ -153,7 +153,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">28</t>
+          <t xml:space="preserve">29</t>
         </is>
       </c>
     </row>
@@ -2792,22 +2792,22 @@
     <row r="51" ht="44" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-OPEN</t>
+          <t xml:space="preserve">RESP-ST-GRID-POWER</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IG-026</t>
+          <t xml:space="preserve">IG-036</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTTripLatch | vppECMS52GTClosedCommandNative</t>
+          <t xml:space="preserve">vpp52STClosed</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52GTClosed</t>
+          <t xml:space="preserve">vppSTGridPowerMW</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -2837,29 +2837,29 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
+          <t xml:space="preserve">SEQ-52GT-OPEN</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IG-025</t>
+          <t xml:space="preserve">IG-026</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTTripLatch</t>
+          <t xml:space="preserve">vppGTTripLatch | vppECMS52GTClosedCommandNative</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52GTTripCmd</t>
+          <t xml:space="preserve">vpp52GTClosed</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2896,22 +2896,22 @@
     <row r="53" ht="44" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52ST-OPEN</t>
+          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IG-028</t>
+          <t xml:space="preserve">IG-025</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripLatchPublished | vppECMS52STClosedCommandNative</t>
+          <t xml:space="preserve">vppGTTripLatch</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52STClosed</t>
+          <t xml:space="preserve">vpp52GTTripCmd</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -2948,57 +2948,109 @@
     <row r="54" ht="44" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">SEQ-52ST-OPEN</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IG-028</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vppSTTripLatchPublished | vppECMS52STClosedCommandNative</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vpp52STClosed</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXACT_REGISTERED_IDENTITIES</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LIVE_CENSUS_RESOLVED</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="44" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">SEQ-52ST-TRIPCMD</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">IG-027</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">vppSTTripLatchPublished</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">vpp52STTripCmd</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">EXACT_REGISTERED_IDENTITIES</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr">
+      <c r="I55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">LIVE_CENSUS_RESOLVED</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr">
+      <c r="J55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">PASS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J54"/>
+  <autoFilter ref="A1:J55"/>
 </worksheet>
 </file>
 
@@ -6255,7 +6307,7 @@
     <row r="121" ht="44" customHeight="1">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-OPEN</t>
+          <t xml:space="preserve">RESP-ST-GRID-POWER</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -6270,7 +6322,7 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTTripLatch</t>
+          <t xml:space="preserve">vpp52STClosed</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -6282,22 +6334,22 @@
     <row r="122" ht="44" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-OPEN</t>
+          <t xml:space="preserve">RESP-ST-GRID-POWER</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-02</t>
+          <t xml:space="preserve">OUT-01</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">INPUT</t>
+          <t xml:space="preserve">OUTPUT</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppECMS52GTClosedCommandNative</t>
+          <t xml:space="preserve">vppSTGridPowerMW</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -6314,17 +6366,17 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUT-01</t>
+          <t xml:space="preserve">IN-01</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUTPUT</t>
+          <t xml:space="preserve">INPUT</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52GTClosed</t>
+          <t xml:space="preserve">vppGTTripLatch</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
@@ -6336,12 +6388,12 @@
     <row r="124" ht="44" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
+          <t xml:space="preserve">SEQ-52GT-OPEN</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-01</t>
+          <t xml:space="preserve">IN-02</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -6351,7 +6403,7 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTTripLatch</t>
+          <t xml:space="preserve">vppECMS52GTClosedCommandNative</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -6363,7 +6415,7 @@
     <row r="125" ht="44" customHeight="1">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
+          <t xml:space="preserve">SEQ-52GT-OPEN</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -6378,7 +6430,7 @@
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52GTTripCmd</t>
+          <t xml:space="preserve">vpp52GTClosed</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
@@ -6390,7 +6442,7 @@
     <row r="126" ht="44" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52ST-OPEN</t>
+          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -6405,7 +6457,7 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripLatchPublished</t>
+          <t xml:space="preserve">vppGTTripLatch</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -6417,22 +6469,22 @@
     <row r="127" ht="44" customHeight="1">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52ST-OPEN</t>
+          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-02</t>
+          <t xml:space="preserve">OUT-01</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">INPUT</t>
+          <t xml:space="preserve">OUTPUT</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppECMS52STClosedCommandNative</t>
+          <t xml:space="preserve">vpp52GTTripCmd</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -6449,17 +6501,17 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUT-01</t>
+          <t xml:space="preserve">IN-01</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUTPUT</t>
+          <t xml:space="preserve">INPUT</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52STClosed</t>
+          <t xml:space="preserve">vppSTTripLatchPublished</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -6471,12 +6523,12 @@
     <row r="129" ht="44" customHeight="1">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52ST-TRIPCMD</t>
+          <t xml:space="preserve">SEQ-52ST-OPEN</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-01</t>
+          <t xml:space="preserve">IN-02</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
@@ -6486,7 +6538,7 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripLatchPublished</t>
+          <t xml:space="preserve">vppECMS52STClosedCommandNative</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
@@ -6498,31 +6550,85 @@
     <row r="130" ht="44" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">SEQ-52ST-OPEN</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUT-01</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUTPUT</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vpp52STClosed</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RAW_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="44" customHeight="1">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">SEQ-52ST-TRIPCMD</t>
         </is>
       </c>
-      <c r="B130" s="2" t="inlineStr">
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IN-01</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INPUT</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vppSTTripLatchPublished</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RAW_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="44" customHeight="1">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEQ-52ST-TRIPCMD</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">OUT-01</t>
         </is>
       </c>
-      <c r="C130" s="2" t="inlineStr">
+      <c r="C132" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">OUTPUT</t>
         </is>
       </c>
-      <c r="D130" s="2" t="inlineStr">
+      <c r="D132" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">vpp52STTripCmd</t>
         </is>
       </c>
-      <c r="E130" s="2" t="inlineStr">
+      <c r="E132" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">RAW_NODE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E130"/>
+  <autoFilter ref="A1:E132"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish ST grid power in web masters (#70)
Register vppSTGridPowerMW in the verified TAG, Logic, and Drawing masters; publish a read-only Plant Process navigation link; keep behavior verification PARTIAL and raw plant telemetry private.
</commit_message>
<xml_diff>
--- a/generated/logic/08_TAG_LOGIC_LINK_MASTER_VALIDATION.xlsx
+++ b/generated/logic/08_TAG_LOGIC_LINK_MASTER_VALIDATION.xlsx
@@ -81,7 +81,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">603</t>
+          <t xml:space="preserve">604</t>
         </is>
       </c>
     </row>
@@ -93,7 +93,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">53</t>
+          <t xml:space="preserve">54</t>
         </is>
       </c>
     </row>
@@ -105,7 +105,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">35</t>
+          <t xml:space="preserve">36</t>
         </is>
       </c>
     </row>
@@ -129,7 +129,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">98</t>
+          <t xml:space="preserve">100</t>
         </is>
       </c>
     </row>
@@ -141,7 +141,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">44</t>
+          <t xml:space="preserve">45</t>
         </is>
       </c>
     </row>
@@ -153,7 +153,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">28</t>
+          <t xml:space="preserve">29</t>
         </is>
       </c>
     </row>
@@ -2792,22 +2792,22 @@
     <row r="51" ht="44" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-OPEN</t>
+          <t xml:space="preserve">RESP-ST-GRID-POWER</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IG-026</t>
+          <t xml:space="preserve">IG-036</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTTripLatch | vppECMS52GTClosedCommandNative</t>
+          <t xml:space="preserve">vpp52STClosed</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52GTClosed</t>
+          <t xml:space="preserve">vppSTGridPowerMW</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -2837,29 +2837,29 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
+          <t xml:space="preserve">SEQ-52GT-OPEN</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IG-025</t>
+          <t xml:space="preserve">IG-026</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTTripLatch</t>
+          <t xml:space="preserve">vppGTTripLatch | vppECMS52GTClosedCommandNative</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52GTTripCmd</t>
+          <t xml:space="preserve">vpp52GTClosed</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2896,22 +2896,22 @@
     <row r="53" ht="44" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52ST-OPEN</t>
+          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IG-028</t>
+          <t xml:space="preserve">IG-025</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripLatchPublished | vppECMS52STClosedCommandNative</t>
+          <t xml:space="preserve">vppGTTripLatch</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52STClosed</t>
+          <t xml:space="preserve">vpp52GTTripCmd</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -2948,57 +2948,109 @@
     <row r="54" ht="44" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">SEQ-52ST-OPEN</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IG-028</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vppSTTripLatchPublished | vppECMS52STClosedCommandNative</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vpp52STClosed</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXACT_REGISTERED_IDENTITIES</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LIVE_CENSUS_RESOLVED</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="44" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">SEQ-52ST-TRIPCMD</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">IG-027</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">vppSTTripLatchPublished</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">vpp52STTripCmd</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">EXACT_REGISTERED_IDENTITIES</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr">
+      <c r="I55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">LIVE_CENSUS_RESOLVED</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr">
+      <c r="J55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">PASS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J54"/>
+  <autoFilter ref="A1:J55"/>
 </worksheet>
 </file>
 
@@ -6255,7 +6307,7 @@
     <row r="121" ht="44" customHeight="1">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-OPEN</t>
+          <t xml:space="preserve">RESP-ST-GRID-POWER</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -6270,7 +6322,7 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTTripLatch</t>
+          <t xml:space="preserve">vpp52STClosed</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -6282,22 +6334,22 @@
     <row r="122" ht="44" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-OPEN</t>
+          <t xml:space="preserve">RESP-ST-GRID-POWER</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-02</t>
+          <t xml:space="preserve">OUT-01</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">INPUT</t>
+          <t xml:space="preserve">OUTPUT</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppECMS52GTClosedCommandNative</t>
+          <t xml:space="preserve">vppSTGridPowerMW</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -6314,17 +6366,17 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUT-01</t>
+          <t xml:space="preserve">IN-01</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUTPUT</t>
+          <t xml:space="preserve">INPUT</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52GTClosed</t>
+          <t xml:space="preserve">vppGTTripLatch</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
@@ -6336,12 +6388,12 @@
     <row r="124" ht="44" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
+          <t xml:space="preserve">SEQ-52GT-OPEN</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-01</t>
+          <t xml:space="preserve">IN-02</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -6351,7 +6403,7 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTTripLatch</t>
+          <t xml:space="preserve">vppECMS52GTClosedCommandNative</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -6363,7 +6415,7 @@
     <row r="125" ht="44" customHeight="1">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
+          <t xml:space="preserve">SEQ-52GT-OPEN</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -6378,7 +6430,7 @@
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52GTTripCmd</t>
+          <t xml:space="preserve">vpp52GTClosed</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
@@ -6390,7 +6442,7 @@
     <row r="126" ht="44" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52ST-OPEN</t>
+          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -6405,7 +6457,7 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripLatchPublished</t>
+          <t xml:space="preserve">vppGTTripLatch</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -6417,22 +6469,22 @@
     <row r="127" ht="44" customHeight="1">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52ST-OPEN</t>
+          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-02</t>
+          <t xml:space="preserve">OUT-01</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">INPUT</t>
+          <t xml:space="preserve">OUTPUT</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppECMS52STClosedCommandNative</t>
+          <t xml:space="preserve">vpp52GTTripCmd</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -6449,17 +6501,17 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUT-01</t>
+          <t xml:space="preserve">IN-01</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUTPUT</t>
+          <t xml:space="preserve">INPUT</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52STClosed</t>
+          <t xml:space="preserve">vppSTTripLatchPublished</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -6471,12 +6523,12 @@
     <row r="129" ht="44" customHeight="1">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52ST-TRIPCMD</t>
+          <t xml:space="preserve">SEQ-52ST-OPEN</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-01</t>
+          <t xml:space="preserve">IN-02</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
@@ -6486,7 +6538,7 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripLatchPublished</t>
+          <t xml:space="preserve">vppECMS52STClosedCommandNative</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
@@ -6498,31 +6550,85 @@
     <row r="130" ht="44" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">SEQ-52ST-OPEN</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUT-01</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUTPUT</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vpp52STClosed</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RAW_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="44" customHeight="1">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">SEQ-52ST-TRIPCMD</t>
         </is>
       </c>
-      <c r="B130" s="2" t="inlineStr">
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IN-01</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INPUT</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vppSTTripLatchPublished</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RAW_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="44" customHeight="1">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEQ-52ST-TRIPCMD</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">OUT-01</t>
         </is>
       </c>
-      <c r="C130" s="2" t="inlineStr">
+      <c r="C132" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">OUTPUT</t>
         </is>
       </c>
-      <c r="D130" s="2" t="inlineStr">
+      <c r="D132" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">vpp52STTripCmd</t>
         </is>
       </c>
-      <c r="E130" s="2" t="inlineStr">
+      <c r="E132" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">RAW_NODE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E130"/>
+  <autoFilter ref="A1:E132"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Separate ST source observations from the live census
</commit_message>
<xml_diff>
--- a/generated/logic/08_TAG_LOGIC_LINK_MASTER_VALIDATION.xlsx
+++ b/generated/logic/08_TAG_LOGIC_LINK_MASTER_VALIDATION.xlsx
@@ -81,96 +81,168 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">605</t>
+          <t xml:space="preserve">603</t>
         </is>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules</t>
+          <t xml:space="preserve">live_tags</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">54</t>
+          <t xml:space="preserve">603</t>
         </is>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">input_groups</t>
+          <t xml:space="preserve">searchable_tags</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">36</t>
+          <t xml:space="preserve">605</t>
         </is>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">equipment_pages</t>
+          <t xml:space="preserve">model_source_raw_observed_tags</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">pages</t>
+          <t xml:space="preserve">rules</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">100</t>
+          <t xml:space="preserve">54</t>
         </is>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">native_inputs</t>
+          <t xml:space="preserve">live_rules</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">46</t>
+          <t xml:space="preserve">53</t>
         </is>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">native_outputs</t>
+          <t xml:space="preserve">source_mapped_rules</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">29</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">input_groups</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">36</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">live_input_groups</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">35</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">equipment_pages</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pages</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="44" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">native_inputs</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">46</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="44" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">native_outputs</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">29</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">derived_outputs</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">28</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B15"/>
 </worksheet>
 </file>
 
@@ -2802,7 +2874,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52STClosed | vppSTGeneratorPowerMW</t>
+          <t xml:space="preserve">vppSTGeneratorPowerMW | vpp52STClosed</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2827,12 +2899,12 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXACT_REGISTERED_IDENTITIES</t>
+          <t xml:space="preserve">SOURCE_MAPPED_ONLY</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LIVE_CENSUS_RESOLVED</t>
+          <t xml:space="preserve">MODEL_SOURCE_CONFIRMED_RAW_OBSERVED</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
@@ -6322,12 +6394,12 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52STClosed</t>
+          <t xml:space="preserve">vppSTGeneratorPowerMW</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RAW_NODE</t>
+          <t xml:space="preserve">MODEL_SOURCE_RAW_OBSERVED</t>
         </is>
       </c>
     </row>
@@ -6349,7 +6421,7 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTGeneratorPowerMW</t>
+          <t xml:space="preserve">vpp52STClosed</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -6381,7 +6453,7 @@
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RAW_NODE</t>
+          <t xml:space="preserve">MODEL_SOURCE_RAW_OBSERVED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ST breaker-open Logic and Drawing Master
Add the verified 52ST manual-open protection cause, retire fixed cause-count wording, publish regenerated Logic/Drawing Master assets, and promote the verified ST grid-power OPEN response.
</commit_message>
<xml_diff>
--- a/generated/logic/08_TAG_LOGIC_LINK_MASTER_VALIDATION.xlsx
+++ b/generated/logic/08_TAG_LOGIC_LINK_MASTER_VALIDATION.xlsx
@@ -81,96 +81,168 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">604</t>
+          <t xml:space="preserve">603</t>
         </is>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules</t>
+          <t xml:space="preserve">live_tags</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">54</t>
+          <t xml:space="preserve">603</t>
         </is>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">input_groups</t>
+          <t xml:space="preserve">searchable_tags</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">36</t>
+          <t xml:space="preserve">606</t>
         </is>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">equipment_pages</t>
+          <t xml:space="preserve">model_source_raw_observed_tags</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">pages</t>
+          <t xml:space="preserve">rules</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">100</t>
+          <t xml:space="preserve">55</t>
         </is>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">native_inputs</t>
+          <t xml:space="preserve">live_rules</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">45</t>
+          <t xml:space="preserve">53</t>
         </is>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">native_outputs</t>
+          <t xml:space="preserve">source_mapped_rules</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">29</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">input_groups</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">37</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">live_input_groups</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">35</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">equipment_pages</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pages</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">102</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="44" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">native_inputs</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">47</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="44" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">native_outputs</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">derived_outputs</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">28</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B15"/>
 </worksheet>
 </file>
 
@@ -2584,22 +2656,22 @@
     <row r="47" ht="44" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROT-ST-LATCH</t>
+          <t xml:space="preserve">PROT-ST-BRK-OPEN</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IG-024</t>
+          <t xml:space="preserve">IG-037</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripRequest | vppSTTripResetNative</t>
+          <t xml:space="preserve">vppECMS52STClosedCommandNative</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripLatchPublished</t>
+          <t xml:space="preserve">vppCauseSTBreakerOpenWhileRunning</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2619,12 +2691,12 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXACT_REGISTERED_IDENTITIES</t>
+          <t xml:space="preserve">SOURCE_MAPPED_ONLY</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LIVE_CENSUS_RESOLVED</t>
+          <t xml:space="preserve">MODEL_SOURCE_RUNTIME_VERIFIED</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -2636,22 +2708,22 @@
     <row r="48" ht="44" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROT-ST-REQUEST</t>
+          <t xml:space="preserve">PROT-ST-LATCH</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IG-022</t>
+          <t xml:space="preserve">IG-024</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppCauseDirectGTTrip | vppCauseDirectSTTrip | vppCauseGTBreakerOpenWhileRunning | vppCauseHPDrumHH | vppCauseIPDrumHH | vppCauseLPDrumHH | vppCauseHPDrumLL | vppCauseIPDrumLL | vppCauseLPDrumLL</t>
+          <t xml:space="preserve">vppSTTripRequest | vppSTTripResetNative</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripRequest</t>
+          <t xml:space="preserve">vppSTTripLatchPublished</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2688,22 +2760,22 @@
     <row r="49" ht="44" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RESP-GT-POWER</t>
+          <t xml:space="preserve">PROT-ST-REQUEST</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IG-029</t>
+          <t xml:space="preserve">IG-022</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52GTClosed</t>
+          <t xml:space="preserve">vppGTTripRequest | vppCauseDirectSTTrip | vppCauseSTBreakerOpenWhileRunning | vppCauseHPDrumHH | vppCauseIPDrumHH | vppCauseLPDrumHH</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTGPowerMW</t>
+          <t xml:space="preserve">vppSTTripRequest</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -2723,12 +2795,12 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXACT_REGISTERED_IDENTITIES</t>
+          <t xml:space="preserve">SOURCE_MAPPED_ONLY</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LIVE_CENSUS_RESOLVED</t>
+          <t xml:space="preserve">MODEL_SOURCE_RUNTIME_VERIFIED</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -2740,7 +2812,7 @@
     <row r="50" ht="44" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RESP-GT-SPEED</t>
+          <t xml:space="preserve">RESP-GT-POWER</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2755,7 +2827,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTGSpeedRPM</t>
+          <t xml:space="preserve">vppGTGPowerMW</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2792,22 +2864,22 @@
     <row r="51" ht="44" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RESP-ST-GRID-POWER</t>
+          <t xml:space="preserve">RESP-GT-SPEED</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IG-036</t>
+          <t xml:space="preserve">IG-029</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52STClosed</t>
+          <t xml:space="preserve">vpp52GTClosed</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTGridPowerMW</t>
+          <t xml:space="preserve">vppGTGSpeedRPM</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -2837,29 +2909,29 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PARTIAL</t>
+          <t xml:space="preserve">PASS</t>
         </is>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-OPEN</t>
+          <t xml:space="preserve">RESP-ST-GRID-POWER</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IG-026</t>
+          <t xml:space="preserve">IG-036</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTTripLatch | vppECMS52GTClosedCommandNative</t>
+          <t xml:space="preserve">vppSTGeneratorPowerMW | vpp52STClosed</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52GTClosed</t>
+          <t xml:space="preserve">vppSTGridPowerMW</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2879,12 +2951,12 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXACT_REGISTERED_IDENTITIES</t>
+          <t xml:space="preserve">SOURCE_MAPPED_ONLY</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LIVE_CENSUS_RESOLVED</t>
+          <t xml:space="preserve">MODEL_SOURCE_RUNTIME_VERIFIED</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -2896,22 +2968,22 @@
     <row r="53" ht="44" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
+          <t xml:space="preserve">SEQ-52GT-OPEN</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IG-025</t>
+          <t xml:space="preserve">IG-026</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTTripLatch</t>
+          <t xml:space="preserve">vppGTTripLatch | vppECMS52GTClosedCommandNative</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52GTTripCmd</t>
+          <t xml:space="preserve">vpp52GTClosed</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -2948,22 +3020,22 @@
     <row r="54" ht="44" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEQ-52ST-OPEN</t>
+          <t xml:space="preserve">SEQ-52GT-TRIPCMD</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IG-028</t>
+          <t xml:space="preserve">IG-025</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripLatchPublished | vppECMS52STClosedCommandNative</t>
+          <t xml:space="preserve">vppGTTripLatch</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52STClosed</t>
+          <t xml:space="preserve">vpp52GTTripCmd</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -3000,57 +3072,109 @@
     <row r="55" ht="44" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">SEQ-52ST-OPEN</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IG-028</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vppSTTripLatchPublished | vppECMS52STClosedCommandNative</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vpp52STClosed</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXACT_REGISTERED_IDENTITIES</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LIVE_CENSUS_RESOLVED</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="44" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">SEQ-52ST-TRIPCMD</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">IG-027</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">vppSTTripLatchPublished</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">vpp52STTripCmd</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">EXACT_REGISTERED_IDENTITIES</t>
         </is>
       </c>
-      <c r="I55" s="2" t="inlineStr">
+      <c r="I56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">LIVE_CENSUS_RESOLVED</t>
         </is>
       </c>
-      <c r="J55" s="2" t="inlineStr">
+      <c r="J56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">PASS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J55"/>
+  <autoFilter ref="A1:J56"/>
 </worksheet>
 </file>
 
@@ -5848,7 +5972,7 @@
     <row r="104" ht="44" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROT-ST-LATCH</t>
+          <t xml:space="preserve">PROT-ST-BRK-OPEN</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -5863,7 +5987,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripRequest</t>
+          <t xml:space="preserve">vppECMS52STClosedCommandNative</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -5875,27 +5999,27 @@
     <row r="105" ht="44" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROT-ST-LATCH</t>
+          <t xml:space="preserve">PROT-ST-BRK-OPEN</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-02</t>
+          <t xml:space="preserve">OUT-01</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">INPUT</t>
+          <t xml:space="preserve">OUTPUT</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripResetNative</t>
+          <t xml:space="preserve">vppCauseSTBreakerOpenWhileRunning</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RAW_NODE</t>
+          <t xml:space="preserve">MODEL_SOURCE_RAW_OBSERVED</t>
         </is>
       </c>
     </row>
@@ -5907,17 +6031,17 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUT-01</t>
+          <t xml:space="preserve">IN-01</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUTPUT</t>
+          <t xml:space="preserve">INPUT</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripLatchPublished</t>
+          <t xml:space="preserve">vppSTTripRequest</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -5929,12 +6053,12 @@
     <row r="107" ht="44" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROT-ST-REQUEST</t>
+          <t xml:space="preserve">PROT-ST-LATCH</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-01</t>
+          <t xml:space="preserve">IN-02</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
@@ -5944,7 +6068,7 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppCauseDirectGTTrip</t>
+          <t xml:space="preserve">vppSTTripResetNative</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -5956,22 +6080,22 @@
     <row r="108" ht="44" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROT-ST-REQUEST</t>
+          <t xml:space="preserve">PROT-ST-LATCH</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-02</t>
+          <t xml:space="preserve">OUT-01</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">INPUT</t>
+          <t xml:space="preserve">OUTPUT</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppCauseDirectSTTrip</t>
+          <t xml:space="preserve">vppSTTripLatchPublished</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -5988,7 +6112,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-03</t>
+          <t xml:space="preserve">IN-01</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -5998,7 +6122,7 @@
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppCauseGTBreakerOpenWhileRunning</t>
+          <t xml:space="preserve">vppGTTripRequest</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
@@ -6015,7 +6139,7 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-04</t>
+          <t xml:space="preserve">IN-02</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -6025,7 +6149,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppCauseHPDrumHH</t>
+          <t xml:space="preserve">vppCauseDirectSTTrip</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -6042,7 +6166,7 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-05</t>
+          <t xml:space="preserve">IN-03</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
@@ -6052,12 +6176,12 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppCauseIPDrumHH</t>
+          <t xml:space="preserve">vppCauseSTBreakerOpenWhileRunning</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RAW_NODE</t>
+          <t xml:space="preserve">MODEL_SOURCE_RAW_OBSERVED</t>
         </is>
       </c>
     </row>
@@ -6069,7 +6193,7 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-06</t>
+          <t xml:space="preserve">IN-04</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
@@ -6079,7 +6203,7 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppCauseLPDrumHH</t>
+          <t xml:space="preserve">vppCauseHPDrumHH</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -6096,7 +6220,7 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-07</t>
+          <t xml:space="preserve">IN-05</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -6106,7 +6230,7 @@
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppCauseHPDrumLL</t>
+          <t xml:space="preserve">vppCauseIPDrumHH</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
@@ -6123,7 +6247,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-08</t>
+          <t xml:space="preserve">IN-06</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -6133,7 +6257,7 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppCauseIPDrumLL</t>
+          <t xml:space="preserve">vppCauseLPDrumHH</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -6150,17 +6274,17 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-09</t>
+          <t xml:space="preserve">OUT-01</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">INPUT</t>
+          <t xml:space="preserve">OUTPUT</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppCauseLPDrumLL</t>
+          <t xml:space="preserve">vppSTTripRequest</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
@@ -6172,22 +6296,22 @@
     <row r="116" ht="44" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROT-ST-REQUEST</t>
+          <t xml:space="preserve">RESP-GT-POWER</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUT-01</t>
+          <t xml:space="preserve">IN-01</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUTPUT</t>
+          <t xml:space="preserve">INPUT</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppSTTripRequest</t>
+          <t xml:space="preserve">vpp52GTClosed</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -6204,17 +6328,17 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-01</t>
+          <t xml:space="preserve">OUT-01</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">INPUT</t>
+          <t xml:space="preserve">OUTPUT</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52GTClosed</t>
+          <t xml:space="preserve">vppGTGPowerMW</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
@@ -6226,22 +6350,22 @@
     <row r="118" ht="44" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RESP-GT-POWER</t>
+          <t xml:space="preserve">RESP-GT-SPEED</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUT-01</t>
+          <t xml:space="preserve">IN-01</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUTPUT</t>
+          <t xml:space="preserve">INPUT</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTGPowerMW</t>
+          <t xml:space="preserve">vpp52GTClosed</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -6258,17 +6382,17 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-01</t>
+          <t xml:space="preserve">OUT-01</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">INPUT</t>
+          <t xml:space="preserve">OUTPUT</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vpp52GTClosed</t>
+          <t xml:space="preserve">vppGTGSpeedRPM</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
@@ -6280,27 +6404,27 @@
     <row r="120" ht="44" customHeight="1">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RESP-GT-SPEED</t>
+          <t xml:space="preserve">RESP-ST-GRID-POWER</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUT-01</t>
+          <t xml:space="preserve">IN-01</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUTPUT</t>
+          <t xml:space="preserve">INPUT</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vppGTGSpeedRPM</t>
+          <t xml:space="preserve">vppSTGeneratorPowerMW</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RAW_NODE</t>
+          <t xml:space="preserve">MODEL_SOURCE_RAW_OBSERVED</t>
         </is>
       </c>
     </row>
@@ -6312,7 +6436,7 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN-01</t>
+          <t xml:space="preserve">IN-02</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
@@ -6354,7 +6478,7 @@
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RAW_NODE</t>
+          <t xml:space="preserve">MODEL_SOURCE_RAW_OBSERVED</t>
         </is>
       </c>
     </row>

</xml_diff>